<commit_message>
List CV entries oldest first in cv.xlsx; show them newest first
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/cv/cv.xlsx
+++ b/cv/cv.xlsx
@@ -747,7 +747,7 @@
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>How to use: sections appear in this order. type = list (rows in the sheet with the same name) or text (the text column). web/pdf = yes/no. details_in_pdf = no hides the details column in the PDF (e.g. talk titles).</t>
+          <t>How to use: sections appear in this order. type = list (rows in the sheet with the same name) or text (the text column). web/pdf = yes/no. details_in_pdf = no hides the details column in the PDF (e.g. talk titles). In the other sheets, put older entries first and add new ones at the bottom; the CV shows them newest first.</t>
         </is>
       </c>
       <c r="B12" s="2" t="n"/>
@@ -845,118 +845,118 @@
     <row r="2">
       <c r="A2" s="3" t="inlineStr">
         <is>
-          <t>2023–Present</t>
+          <t>2017–2021</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>PhD Researcher</t>
-        </is>
-      </c>
-      <c r="C2" s="2" t="inlineStr"/>
+          <t>Degree in Mathematics</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="n"/>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>Basque Center for Applied Mathematics (BCAM)</t>
-        </is>
-      </c>
-      <c r="E2" s="2" t="inlineStr"/>
+          <t>Universidad Complutense de Madrid</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="n"/>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>Bilbao, Spain</t>
-        </is>
-      </c>
-      <c r="G2" s="2" t="inlineStr">
-        <is>
-          <t>Supervisor: Ilya Smirnov.</t>
-        </is>
-      </c>
-      <c r="H2" s="2" t="inlineStr"/>
-      <c r="I2" s="2" t="inlineStr"/>
-      <c r="J2" s="2" t="inlineStr"/>
+          <t>Madrid, Spain</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="n"/>
+      <c r="H2" s="2" t="n"/>
+      <c r="I2" s="2" t="n"/>
+      <c r="J2" s="2" t="n"/>
     </row>
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>Fall 2022</t>
+          <t>2021–2022</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Research Internship</t>
-        </is>
-      </c>
-      <c r="C3" s="2" t="inlineStr"/>
+          <t>Master's Degree in Advanced Mathematics</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="n"/>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>BCAM</t>
-        </is>
-      </c>
-      <c r="E3" s="2" t="inlineStr"/>
+          <t>Universidad Complutense de Madrid</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="n"/>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>Bilbao, Spain</t>
-        </is>
-      </c>
-      <c r="G3" s="2" t="inlineStr"/>
-      <c r="H3" s="2" t="inlineStr"/>
-      <c r="I3" s="2" t="inlineStr"/>
-      <c r="J3" s="2" t="inlineStr"/>
+          <t>Madrid, Spain</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="n"/>
+      <c r="H3" s="2" t="n"/>
+      <c r="I3" s="2" t="n"/>
+      <c r="J3" s="2" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>2021–2022</t>
+          <t>Fall 2022</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Master's Degree in Advanced Mathematics</t>
-        </is>
-      </c>
-      <c r="C4" s="2" t="inlineStr"/>
+          <t>Research Internship</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="n"/>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>Universidad Complutense de Madrid</t>
-        </is>
-      </c>
-      <c r="E4" s="2" t="inlineStr"/>
+          <t>BCAM</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="n"/>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Madrid, Spain</t>
-        </is>
-      </c>
-      <c r="G4" s="2" t="inlineStr"/>
-      <c r="H4" s="2" t="inlineStr"/>
-      <c r="I4" s="2" t="inlineStr"/>
-      <c r="J4" s="2" t="inlineStr"/>
+          <t>Bilbao, Spain</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="n"/>
+      <c r="H4" s="2" t="n"/>
+      <c r="I4" s="2" t="n"/>
+      <c r="J4" s="2" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>2017–2021</t>
+          <t>2023–Present</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Degree in Mathematics</t>
-        </is>
-      </c>
-      <c r="C5" s="2" t="inlineStr"/>
+          <t>PhD Researcher</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="n"/>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>Universidad Complutense de Madrid</t>
-        </is>
-      </c>
-      <c r="E5" s="2" t="inlineStr"/>
+          <t>Basque Center for Applied Mathematics (BCAM)</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="n"/>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>Madrid, Spain</t>
-        </is>
-      </c>
-      <c r="G5" s="2" t="inlineStr"/>
-      <c r="H5" s="2" t="inlineStr"/>
-      <c r="I5" s="2" t="inlineStr"/>
-      <c r="J5" s="2" t="inlineStr"/>
+          <t>Bilbao, Spain</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t>Supervisor: Ilya Smirnov.</t>
+        </is>
+      </c>
+      <c r="H5" s="2" t="n"/>
+      <c r="I5" s="2" t="n"/>
+      <c r="J5" s="2" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="3" t="n"/>
@@ -3402,12 +3402,12 @@
           <t>preprint, arXiv</t>
         </is>
       </c>
-      <c r="E2" s="2" t="inlineStr"/>
-      <c r="F2" s="2" t="inlineStr"/>
-      <c r="G2" s="2" t="inlineStr"/>
-      <c r="H2" s="2" t="inlineStr"/>
-      <c r="I2" s="2" t="inlineStr"/>
-      <c r="J2" s="2" t="inlineStr"/>
+      <c r="E2" s="2" t="n"/>
+      <c r="F2" s="2" t="n"/>
+      <c r="G2" s="2" t="n"/>
+      <c r="H2" s="2" t="n"/>
+      <c r="I2" s="2" t="n"/>
+      <c r="J2" s="2" t="n"/>
     </row>
     <row r="3">
       <c r="A3" s="3" t="n"/>
@@ -5871,206 +5871,206 @@
     <row r="2">
       <c r="A2" s="3" t="inlineStr">
         <is>
-          <t>Nov 2025</t>
+          <t>Sep 2022</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>University of Michigan</t>
-        </is>
-      </c>
-      <c r="C2" s="2" t="inlineStr"/>
+          <t>Universidad Complutense de Madrid</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="n"/>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>CA Seminar</t>
-        </is>
-      </c>
-      <c r="E2" s="2" t="inlineStr">
-        <is>
-          <t>https://lsa.umich.edu/math/news-events/all-events.detail.html/142145-21890070.html</t>
-        </is>
-      </c>
+          <t>XVI Workshop de Jóvenes Investigadores</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="n"/>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>Michigan, USA</t>
+          <t>Madrid, Spain</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>*On the Strong Watanabe–Yoshida conjecture*.</t>
-        </is>
-      </c>
-      <c r="H2" s="2" t="inlineStr"/>
-      <c r="I2" s="2" t="inlineStr"/>
-      <c r="J2" s="2" t="inlineStr"/>
+          <t>*The 2875 lines within a general quintic hypersurface of projective 4-space*.</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="n"/>
+      <c r="I2" s="2" t="n"/>
+      <c r="J2" s="2" t="n"/>
     </row>
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>Nov 2025</t>
+          <t>Nov 2023</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>University of Illinois in Chicago</t>
-        </is>
-      </c>
-      <c r="C3" s="2" t="inlineStr"/>
+          <t>ICMAT</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="n"/>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>AG Seminar</t>
-        </is>
-      </c>
-      <c r="E3" s="2" t="inlineStr">
-        <is>
-          <t>https://www.math.uic.edu/persisting_utilities/seminars/view_seminar?id=8039</t>
-        </is>
-      </c>
+          <t>5th BYMAT Conference</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="n"/>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>Illinois, USA</t>
-        </is>
-      </c>
-      <c r="G3" s="2" t="inlineStr">
-        <is>
-          <t>*The Strong Watanabe–Yoshida conjecture for complete intersections*.</t>
-        </is>
-      </c>
-      <c r="H3" s="2" t="inlineStr"/>
-      <c r="I3" s="2" t="inlineStr"/>
-      <c r="J3" s="2" t="inlineStr"/>
+          <t>Madrid, Spain</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="n"/>
+      <c r="H3" s="2" t="n"/>
+      <c r="I3" s="2" t="n"/>
+      <c r="J3" s="2" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>Oct 2025</t>
+          <t>Jan 2024</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Purdue University</t>
-        </is>
-      </c>
-      <c r="C4" s="2" t="inlineStr"/>
+          <t>Universidad de Sevilla</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="n"/>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>CA Seminar</t>
+          <t>RGAS School on Singularities</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>https://vaibhav-pandey1.github.io/seminar.html</t>
+          <t>https://sites.google.com/view/sevillargas/program</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Indiana, USA</t>
+          <t>Seville, Spain</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>*The Strong Watanabe–Yoshida conjecture for complete intersections*.</t>
-        </is>
-      </c>
-      <c r="H4" s="2" t="inlineStr"/>
-      <c r="I4" s="2" t="inlineStr"/>
-      <c r="J4" s="2" t="inlineStr"/>
+          <t>*Hilbert–Kunz theory in characteristic 2*.</t>
+        </is>
+      </c>
+      <c r="H4" s="2" t="n"/>
+      <c r="I4" s="2" t="n"/>
+      <c r="J4" s="2" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>Jan 2024</t>
+          <t>Oct 2025</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Universidad de Sevilla</t>
-        </is>
-      </c>
-      <c r="C5" s="2" t="inlineStr"/>
+          <t>Purdue University</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="n"/>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>RGAS School on Singularities</t>
+          <t>CA Seminar</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>https://sites.google.com/view/sevillargas/program</t>
+          <t>https://vaibhav-pandey1.github.io/seminar.html</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>Seville, Spain</t>
+          <t>Indiana, USA</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>*Hilbert–Kunz theory in characteristic 2*.</t>
-        </is>
-      </c>
-      <c r="H5" s="2" t="inlineStr"/>
-      <c r="I5" s="2" t="inlineStr"/>
-      <c r="J5" s="2" t="inlineStr"/>
+          <t>*The Strong Watanabe–Yoshida conjecture for complete intersections*.</t>
+        </is>
+      </c>
+      <c r="H5" s="2" t="n"/>
+      <c r="I5" s="2" t="n"/>
+      <c r="J5" s="2" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
         <is>
-          <t>Nov 2023</t>
+          <t>Nov 2025</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>ICMAT</t>
-        </is>
-      </c>
-      <c r="C6" s="2" t="inlineStr"/>
+          <t>University of Illinois in Chicago</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="n"/>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>5th BYMAT Conference</t>
-        </is>
-      </c>
-      <c r="E6" s="2" t="inlineStr"/>
+          <t>AG Seminar</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>https://www.math.uic.edu/persisting_utilities/seminars/view_seminar?id=8039</t>
+        </is>
+      </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>Madrid, Spain</t>
-        </is>
-      </c>
-      <c r="G6" s="2" t="inlineStr"/>
-      <c r="H6" s="2" t="inlineStr"/>
-      <c r="I6" s="2" t="inlineStr"/>
-      <c r="J6" s="2" t="inlineStr"/>
+          <t>Illinois, USA</t>
+        </is>
+      </c>
+      <c r="G6" s="2" t="inlineStr">
+        <is>
+          <t>*The Strong Watanabe–Yoshida conjecture for complete intersections*.</t>
+        </is>
+      </c>
+      <c r="H6" s="2" t="n"/>
+      <c r="I6" s="2" t="n"/>
+      <c r="J6" s="2" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t>Sep 2022</t>
+          <t>Nov 2025</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>Universidad Complutense de Madrid</t>
-        </is>
-      </c>
-      <c r="C7" s="2" t="inlineStr"/>
+          <t>University of Michigan</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="n"/>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>XVI Workshop de Jóvenes Investigadores</t>
-        </is>
-      </c>
-      <c r="E7" s="2" t="inlineStr"/>
+          <t>CA Seminar</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>https://lsa.umich.edu/math/news-events/all-events.detail.html/142145-21890070.html</t>
+        </is>
+      </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>Madrid, Spain</t>
+          <t>Michigan, USA</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t>*The 2875 lines within a general quintic hypersurface of projective 4-space*.</t>
-        </is>
-      </c>
-      <c r="H7" s="2" t="inlineStr"/>
-      <c r="I7" s="2" t="inlineStr"/>
-      <c r="J7" s="2" t="inlineStr"/>
+          <t>*On the Strong Watanabe–Yoshida conjecture*.</t>
+        </is>
+      </c>
+      <c r="H7" s="2" t="n"/>
+      <c r="I7" s="2" t="n"/>
+      <c r="J7" s="2" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="3" t="n"/>
@@ -8482,13 +8482,13 @@
           <t>Research Stay</t>
         </is>
       </c>
-      <c r="C2" s="2" t="inlineStr"/>
+      <c r="C2" s="2" t="n"/>
       <c r="D2" s="2" t="inlineStr">
         <is>
           <t>Purdue University</t>
         </is>
       </c>
-      <c r="E2" s="2" t="inlineStr"/>
+      <c r="E2" s="2" t="n"/>
       <c r="F2" s="2" t="inlineStr">
         <is>
           <t>Indiana, USA</t>
@@ -8499,9 +8499,9 @@
           <t>Host: Uli Walther</t>
         </is>
       </c>
-      <c r="H2" s="2" t="inlineStr"/>
-      <c r="I2" s="2" t="inlineStr"/>
-      <c r="J2" s="2" t="inlineStr"/>
+      <c r="H2" s="2" t="n"/>
+      <c r="I2" s="2" t="n"/>
+      <c r="J2" s="2" t="n"/>
     </row>
     <row r="3">
       <c r="A3" s="3" t="n"/>
@@ -10983,7 +10983,7 @@
           <t>Guanajuato</t>
         </is>
       </c>
-      <c r="E2" s="2" t="inlineStr"/>
+      <c r="E2" s="2" t="n"/>
       <c r="F2" s="2" t="inlineStr">
         <is>
           <t>Mexico</t>
@@ -10999,8 +10999,8 @@
           <t>https://sites.google.com/view/singularitiesalggeom2025/poster-session</t>
         </is>
       </c>
-      <c r="I2" s="2" t="inlineStr"/>
-      <c r="J2" s="2" t="inlineStr"/>
+      <c r="I2" s="2" t="n"/>
+      <c r="J2" s="2" t="n"/>
     </row>
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
@@ -11023,7 +11023,7 @@
           <t>Milan</t>
         </is>
       </c>
-      <c r="E3" s="2" t="inlineStr"/>
+      <c r="E3" s="2" t="n"/>
       <c r="F3" s="2" t="inlineStr">
         <is>
           <t>Italy</t>
@@ -11039,8 +11039,8 @@
           <t>https://www.caag26.polimi.it/posters/mudrak/</t>
         </is>
       </c>
-      <c r="I3" s="2" t="inlineStr"/>
-      <c r="J3" s="2" t="inlineStr"/>
+      <c r="I3" s="2" t="n"/>
+      <c r="J3" s="2" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="3" t="n"/>
@@ -13500,22 +13500,22 @@
           <t>Organizer of Parallel Session AL07 “Singularity Theory”</t>
         </is>
       </c>
-      <c r="C2" s="2" t="inlineStr"/>
+      <c r="C2" s="2" t="n"/>
       <c r="D2" s="2" t="inlineStr">
         <is>
           <t>VII Congreso de Jóvenes Investigadores de la RSME (University of the Basque Country)</t>
         </is>
       </c>
-      <c r="E2" s="2" t="inlineStr"/>
+      <c r="E2" s="2" t="n"/>
       <c r="F2" s="2" t="inlineStr">
         <is>
           <t>Bilbao, Spain</t>
         </is>
       </c>
-      <c r="G2" s="2" t="inlineStr"/>
-      <c r="H2" s="2" t="inlineStr"/>
-      <c r="I2" s="2" t="inlineStr"/>
-      <c r="J2" s="2" t="inlineStr"/>
+      <c r="G2" s="2" t="n"/>
+      <c r="H2" s="2" t="n"/>
+      <c r="I2" s="2" t="n"/>
+      <c r="J2" s="2" t="n"/>
     </row>
     <row r="3">
       <c r="A3" s="3" t="n"/>
@@ -15987,22 +15987,22 @@
           <t>*Prehistory of Commutative Algebra: Noether, Hilbert and Noether*</t>
         </is>
       </c>
-      <c r="C2" s="2" t="inlineStr"/>
+      <c r="C2" s="2" t="n"/>
       <c r="D2" s="2" t="inlineStr">
         <is>
           <t>BCAM</t>
         </is>
       </c>
-      <c r="E2" s="2" t="inlineStr"/>
+      <c r="E2" s="2" t="n"/>
       <c r="F2" s="2" t="inlineStr">
         <is>
           <t>Bilbao, Spain</t>
         </is>
       </c>
-      <c r="G2" s="2" t="inlineStr"/>
-      <c r="H2" s="2" t="inlineStr"/>
-      <c r="I2" s="2" t="inlineStr"/>
-      <c r="J2" s="2" t="inlineStr"/>
+      <c r="G2" s="2" t="n"/>
+      <c r="H2" s="2" t="n"/>
+      <c r="I2" s="2" t="n"/>
+      <c r="J2" s="2" t="n"/>
     </row>
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
@@ -16015,22 +16015,22 @@
           <t>*F-invariants and F-singularities, interactions*</t>
         </is>
       </c>
-      <c r="C3" s="2" t="inlineStr"/>
+      <c r="C3" s="2" t="n"/>
       <c r="D3" s="2" t="inlineStr">
         <is>
           <t>Purdue Grad student seminar</t>
         </is>
       </c>
-      <c r="E3" s="2" t="inlineStr"/>
+      <c r="E3" s="2" t="n"/>
       <c r="F3" s="2" t="inlineStr">
         <is>
           <t>Indiana, USA</t>
         </is>
       </c>
-      <c r="G3" s="2" t="inlineStr"/>
-      <c r="H3" s="2" t="inlineStr"/>
-      <c r="I3" s="2" t="inlineStr"/>
-      <c r="J3" s="2" t="inlineStr"/>
+      <c r="G3" s="2" t="n"/>
+      <c r="H3" s="2" t="n"/>
+      <c r="I3" s="2" t="n"/>
+      <c r="J3" s="2" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="3" t="n"/>
@@ -18482,174 +18482,174 @@
     <row r="2">
       <c r="A2" s="3" t="inlineStr">
         <is>
-          <t>Oct 2025</t>
+          <t>Nov 2022</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>KUMUNU 2025</t>
-        </is>
-      </c>
-      <c r="C2" s="2" t="inlineStr">
-        <is>
-          <t>https://sites.google.com/view/kumunu2025/home</t>
-        </is>
-      </c>
+          <t>BCAM-Severo Ochoa Lecture: Introduction to Morse Homology</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="n"/>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>University of Missouri</t>
-        </is>
-      </c>
-      <c r="E2" s="2" t="inlineStr"/>
+          <t>Bilbao</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="n"/>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>Columbia, USA</t>
-        </is>
-      </c>
-      <c r="G2" s="2" t="inlineStr"/>
-      <c r="H2" s="2" t="inlineStr"/>
-      <c r="I2" s="2" t="inlineStr"/>
-      <c r="J2" s="2" t="inlineStr"/>
+          <t>Spain</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="n"/>
+      <c r="H2" s="2" t="n"/>
+      <c r="I2" s="2" t="n"/>
+      <c r="J2" s="2" t="n"/>
     </row>
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>Nov 2023</t>
+          <t>Nov 2022</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>IberoSing International Workshop 2023</t>
-        </is>
-      </c>
-      <c r="C3" s="2" t="inlineStr"/>
+          <t>IberoSing International Workshop 2022</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="n"/>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>Granada</t>
-        </is>
-      </c>
-      <c r="E3" s="2" t="inlineStr"/>
+          <t>Madrid</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="n"/>
       <c r="F3" s="2" t="inlineStr">
         <is>
           <t>Spain</t>
         </is>
       </c>
-      <c r="G3" s="2" t="inlineStr"/>
-      <c r="H3" s="2" t="inlineStr"/>
-      <c r="I3" s="2" t="inlineStr"/>
-      <c r="J3" s="2" t="inlineStr"/>
+      <c r="G3" s="2" t="n"/>
+      <c r="H3" s="2" t="n"/>
+      <c r="I3" s="2" t="n"/>
+      <c r="J3" s="2" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>Nov 2024</t>
+          <t>Apr 2023</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Sheaf Cohomology Course</t>
-        </is>
-      </c>
-      <c r="C4" s="2" t="inlineStr"/>
+          <t>BCAM-Severo Ochoa Course: Introduction to multiplicity theory</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="n"/>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>Zaragoza</t>
-        </is>
-      </c>
-      <c r="E4" s="2" t="inlineStr"/>
+          <t>Bilbao</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="n"/>
       <c r="F4" s="2" t="inlineStr">
         <is>
           <t>Spain</t>
         </is>
       </c>
-      <c r="G4" s="2" t="inlineStr"/>
-      <c r="H4" s="2" t="inlineStr"/>
-      <c r="I4" s="2" t="inlineStr"/>
-      <c r="J4" s="2" t="inlineStr"/>
+      <c r="G4" s="2" t="n"/>
+      <c r="H4" s="2" t="n"/>
+      <c r="I4" s="2" t="n"/>
+      <c r="J4" s="2" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>Apr 2023</t>
+          <t>Nov 2023</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>BCAM-Severo Ochoa Course: Introduction to multiplicity theory</t>
-        </is>
-      </c>
-      <c r="C5" s="2" t="inlineStr"/>
+          <t>IberoSing International Workshop 2023</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="n"/>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>Bilbao</t>
-        </is>
-      </c>
-      <c r="E5" s="2" t="inlineStr"/>
+          <t>Granada</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="n"/>
       <c r="F5" s="2" t="inlineStr">
         <is>
           <t>Spain</t>
         </is>
       </c>
-      <c r="G5" s="2" t="inlineStr"/>
-      <c r="H5" s="2" t="inlineStr"/>
-      <c r="I5" s="2" t="inlineStr"/>
-      <c r="J5" s="2" t="inlineStr"/>
+      <c r="G5" s="2" t="n"/>
+      <c r="H5" s="2" t="n"/>
+      <c r="I5" s="2" t="n"/>
+      <c r="J5" s="2" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
         <is>
-          <t>Nov 2022</t>
+          <t>Nov 2024</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>IberoSing International Workshop 2022</t>
-        </is>
-      </c>
-      <c r="C6" s="2" t="inlineStr"/>
+          <t>Sheaf Cohomology Course</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="n"/>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>Madrid</t>
-        </is>
-      </c>
-      <c r="E6" s="2" t="inlineStr"/>
+          <t>Zaragoza</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="n"/>
       <c r="F6" s="2" t="inlineStr">
         <is>
           <t>Spain</t>
         </is>
       </c>
-      <c r="G6" s="2" t="inlineStr"/>
-      <c r="H6" s="2" t="inlineStr"/>
-      <c r="I6" s="2" t="inlineStr"/>
-      <c r="J6" s="2" t="inlineStr"/>
+      <c r="G6" s="2" t="n"/>
+      <c r="H6" s="2" t="n"/>
+      <c r="I6" s="2" t="n"/>
+      <c r="J6" s="2" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t>Nov 2022</t>
+          <t>Oct 2025</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>BCAM-Severo Ochoa Lecture: Introduction to Morse Homology</t>
-        </is>
-      </c>
-      <c r="C7" s="2" t="inlineStr"/>
+          <t>KUMUNU 2025</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>https://sites.google.com/view/kumunu2025/home</t>
+        </is>
+      </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>Bilbao</t>
-        </is>
-      </c>
-      <c r="E7" s="2" t="inlineStr"/>
+          <t>University of Missouri</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="n"/>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>Spain</t>
-        </is>
-      </c>
-      <c r="G7" s="2" t="inlineStr"/>
-      <c r="H7" s="2" t="inlineStr"/>
-      <c r="I7" s="2" t="inlineStr"/>
-      <c r="J7" s="2" t="inlineStr"/>
+          <t>Columbia, USA</t>
+        </is>
+      </c>
+      <c r="G7" s="2" t="n"/>
+      <c r="H7" s="2" t="n"/>
+      <c r="I7" s="2" t="n"/>
+      <c r="J7" s="2" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="3" t="n"/>

</xml_diff>

<commit_message>
CV: add limit F-invariants preprint, EPFL talk, Simons school
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/cv/cv.xlsx
+++ b/cv/cv.xlsx
@@ -3410,10 +3410,26 @@
       <c r="J2" s="2" t="n"/>
     </row>
     <row r="3">
-      <c r="A3" s="3" t="n"/>
-      <c r="B3" s="2" t="n"/>
-      <c r="C3" s="2" t="n"/>
-      <c r="D3" s="2" t="n"/>
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>*Limit F-invariants of the simple singularities and the Fermat hypersurfaces*</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>https://arxiv.org/abs/2609.39133</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>preprint, arXiv</t>
+        </is>
+      </c>
       <c r="E3" s="2" t="n"/>
       <c r="F3" s="2" t="n"/>
       <c r="G3" s="2" t="n"/>
@@ -6073,13 +6089,37 @@
       <c r="J7" s="2" t="n"/>
     </row>
     <row r="8">
-      <c r="A8" s="3" t="n"/>
-      <c r="B8" s="2" t="n"/>
+      <c r="A8" s="3" t="inlineStr">
+        <is>
+          <t>Sep 2026</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>EPFL</t>
+        </is>
+      </c>
       <c r="C8" s="2" t="n"/>
-      <c r="D8" s="2" t="n"/>
-      <c r="E8" s="2" t="n"/>
-      <c r="F8" s="2" t="n"/>
-      <c r="G8" s="2" t="n"/>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>Facets of Frobenius derived invariants (Bernoulli Center)</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>https://sites.google.com/view/alapanmukhopadhyay/home/facets-of-frobenius-derived-invariants/schedule</t>
+        </is>
+      </c>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t>Lausanne, Switzerland</t>
+        </is>
+      </c>
+      <c r="G8" s="2" t="inlineStr">
+        <is>
+          <t>*The Hilbert–Kunz multiplicity of diagonal hypersurfaces*.</t>
+        </is>
+      </c>
       <c r="H8" s="2" t="n"/>
       <c r="I8" s="2" t="n"/>
       <c r="J8" s="2" t="n"/>
@@ -18652,12 +18692,32 @@
       <c r="J7" s="2" t="n"/>
     </row>
     <row r="8">
-      <c r="A8" s="3" t="n"/>
-      <c r="B8" s="2" t="n"/>
-      <c r="C8" s="2" t="n"/>
-      <c r="D8" s="2" t="n"/>
+      <c r="A8" s="3" t="inlineStr">
+        <is>
+          <t>Oct 2026</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>Simons School on Higher Dimensional Varieties</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>https://site.pheedloop.com/event/Simonsschoolonhigherdimensionalvarieties/home/</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>Rényi Institute</t>
+        </is>
+      </c>
       <c r="E8" s="2" t="n"/>
-      <c r="F8" s="2" t="n"/>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t>Budapest, Hungary</t>
+        </is>
+      </c>
       <c r="G8" s="2" t="n"/>
       <c r="H8" s="2" t="n"/>
       <c r="I8" s="2" t="n"/>

</xml_diff>

<commit_message>
Top navigation bar instead of the sidebar; tidier CV page
- Header with Research, Math thoughts, CV and About me; contact details
  move to a footer.
- New Math thoughts page listing the posts, with series grouped.
- CV page: Education hidden, secondary sections collapsible
  (web_collapsed column in cv.xlsx).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/cv/cv.xlsx
+++ b/cv/cv.xlsx
@@ -435,7 +435,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G12"/>
+  <dimension ref="A1:H12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -445,6 +445,7 @@
     <col width="7" customWidth="1" min="5" max="5"/>
     <col width="14" customWidth="1" min="6" max="6"/>
     <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="15" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -483,6 +484,11 @@
           <t>contribution</t>
         </is>
       </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>web_collapsed</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -498,17 +504,22 @@
       <c r="C2" s="2" t="inlineStr"/>
       <c r="D2" s="2" t="inlineStr">
         <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
           <t>yes</t>
         </is>
       </c>
-      <c r="E2" s="2" t="inlineStr">
+      <c r="F2" s="2" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
       </c>
-      <c r="F2" s="2" t="inlineStr">
-        <is>
-          <t>yes</t>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>no</t>
         </is>
       </c>
     </row>
@@ -543,6 +554,11 @@
           <t>yes</t>
         </is>
       </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -571,6 +587,11 @@
           <t>yes</t>
         </is>
       </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -604,6 +625,11 @@
           <t>invited talk</t>
         </is>
       </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -632,6 +658,11 @@
           <t>yes</t>
         </is>
       </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -665,6 +696,11 @@
           <t>poster</t>
         </is>
       </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -693,6 +729,11 @@
           <t>yes</t>
         </is>
       </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -726,6 +767,11 @@
           <t>talk</t>
         </is>
       </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -757,6 +803,11 @@
       <c r="G10" t="inlineStr">
         <is>
           <t>attended</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>yes</t>
         </is>
       </c>
     </row>
@@ -771,7 +822,7 @@
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>How to use: sections appear in this order. type = list (rows from the sheet with the same name), text (the text column) or events (rows of the Events sheet with this contribution). web/pdf = yes/no. details_in_pdf = no hides the talk/poster title (or the details column) in the PDF. In the other sheets, put older entries first and add new ones at the bottom; the CV shows them newest first.</t>
+          <t>How to use: sections appear in this order. type = list (rows from the sheet with the same name), text (the text column) or events (rows of the Events sheet with this contribution). web/pdf = yes/no. details_in_pdf = no hides the talk/poster title (or the details column) in the PDF. In the other sheets, put older entries first and add new ones at the bottom; the CV shows them newest first. web_collapsed = yes shows the section on the web page as a collapsible block, closed by default.</t>
         </is>
       </c>
       <c r="B12" s="2" t="n"/>
@@ -781,7 +832,7 @@
       <c r="F12" s="2" t="n"/>
     </row>
   </sheetData>
-  <dataValidations count="3">
+  <dataValidations count="4">
     <dataValidation sqref="D2:F50" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"yes,no"</formula1>
     </dataValidation>
@@ -790,6 +841,9 @@
     </dataValidation>
     <dataValidation sqref="B2:B50" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"list,text,events"</formula1>
+    </dataValidation>
+    <dataValidation sqref="H2:H50" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"yes,no"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
CV: complete the Light PhD Seminar talk at BCAM
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/cv/cv.xlsx
+++ b/cv/cv.xlsx
@@ -8679,10 +8679,14 @@
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
         <is>
-          <t>2024</t>
-        </is>
-      </c>
-      <c r="B9" s="2" t="inlineStr"/>
+          <t>Dec 2024</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>Light PhD Seminars</t>
+        </is>
+      </c>
       <c r="C9" s="2" t="inlineStr"/>
       <c r="D9" s="2" t="inlineStr">
         <is>
@@ -8701,10 +8705,14 @@
       </c>
       <c r="G9" s="2" t="inlineStr">
         <is>
-          <t>*Prehistory of Commutative Algebra: Noether, Hilbert and Noether*</t>
-        </is>
-      </c>
-      <c r="H9" s="2" t="inlineStr"/>
+          <t>*Prehistory of Commutative Algebra. Noether, Hilbert and Noether*.</t>
+        </is>
+      </c>
+      <c r="H9" s="2" t="inlineStr">
+        <is>
+          <t>https://www.bcamath.org/en/light-phd-seminar-prehistory-commutative-algebra-noether-hilbert-and-noether</t>
+        </is>
+      </c>
       <c r="I9" s="2" t="inlineStr"/>
       <c r="J9" s="2" t="inlineStr"/>
     </row>

</xml_diff>

<commit_message>
CV: links, lecturers and dates for the Severo Ochoa courses
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/cv/cv.xlsx
+++ b/cv/cv.xlsx
@@ -8495,7 +8495,7 @@
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>Nov 2022</t>
+          <t>Oct 2022</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
@@ -8503,8 +8503,16 @@
           <t>BCAM-Severo Ochoa Lecture: Introduction to Morse Homology</t>
         </is>
       </c>
-      <c r="C3" s="2" t="inlineStr"/>
-      <c r="D3" s="2" t="inlineStr"/>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>https://www.bcamath.org/en/bcam-severo-ochoa-lecture-introduction-morse-homology</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>BCAM</t>
+        </is>
+      </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
           <t>Bilbao, Spain</t>
@@ -8515,7 +8523,11 @@
           <t>attended</t>
         </is>
       </c>
-      <c r="G3" s="2" t="inlineStr"/>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>Lecturer: María Pe Pereira (Universidad Complutense de Madrid).</t>
+        </is>
+      </c>
       <c r="H3" s="2" t="inlineStr"/>
       <c r="I3" s="2" t="inlineStr"/>
       <c r="J3" s="2" t="inlineStr"/>
@@ -8559,8 +8571,16 @@
           <t>BCAM-Severo Ochoa Course: Introduction to multiplicity theory</t>
         </is>
       </c>
-      <c r="C5" s="2" t="inlineStr"/>
-      <c r="D5" s="2" t="inlineStr"/>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>https://www.bcamath.org/en/bcam-severo-ochoa-course-introduction-multiplicity-theory</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>BCAM</t>
+        </is>
+      </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
           <t>Bilbao, Spain</t>
@@ -8571,7 +8591,11 @@
           <t>attended</t>
         </is>
       </c>
-      <c r="G5" s="2" t="inlineStr"/>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t>Lecturer: Ilya Smirnov (BCAM-Ikerbasque).</t>
+        </is>
+      </c>
       <c r="H5" s="2" t="inlineStr"/>
       <c r="I5" s="2" t="inlineStr"/>
       <c r="J5" s="2" t="inlineStr"/>

</xml_diff>

<commit_message>
CV: links for the IberoSing workshops
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/cv/cv.xlsx
+++ b/cv/cv.xlsx
@@ -8543,7 +8543,11 @@
           <t>IberoSing International Workshop 2022</t>
         </is>
       </c>
-      <c r="C4" s="2" t="inlineStr"/>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>https://eventos.ucm.es/86046/detail/iberosing-international-workshop-2022.html</t>
+        </is>
+      </c>
       <c r="D4" s="2" t="inlineStr"/>
       <c r="E4" s="2" t="inlineStr">
         <is>
@@ -8611,7 +8615,11 @@
           <t>IberoSing International Workshop 2023</t>
         </is>
       </c>
-      <c r="C6" s="2" t="inlineStr"/>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>https://iberosing.github.io/IW23/</t>
+        </is>
+      </c>
       <c r="D6" s="2" t="inlineStr"/>
       <c r="E6" s="2" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Homepage map of affiliations, talks and conferences, built from the CV spreadsheet
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/cv/cv.xlsx
+++ b/cv/cv.xlsx
@@ -13,6 +13,7 @@
     <sheet name="Visits" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="Events" sheetId="5" state="visible" r:id="rId5"/>
     <sheet name="Organization" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Places" sheetId="7" state="visible" r:id="rId9"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -12461,4 +12462,209 @@
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>place</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>lat</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>lon</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Madrid, Spain</t>
+        </is>
+      </c>
+      <c r="B2" s="2">
+        <v>40.4168</v>
+      </c>
+      <c r="C2" s="2">
+        <v>-3.7038</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>Bilbao, Spain</t>
+        </is>
+      </c>
+      <c r="B3" s="2">
+        <v>43.263</v>
+      </c>
+      <c r="C3" s="2">
+        <v>-2.935</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>Granada, Spain</t>
+        </is>
+      </c>
+      <c r="B4" s="2">
+        <v>37.1773</v>
+      </c>
+      <c r="C4" s="2">
+        <v>-3.5986</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>Seville, Spain</t>
+        </is>
+      </c>
+      <c r="B5" s="2">
+        <v>37.3891</v>
+      </c>
+      <c r="C5" s="2">
+        <v>-5.9845</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>Zaragoza, Spain</t>
+        </is>
+      </c>
+      <c r="B6" s="2">
+        <v>41.6488</v>
+      </c>
+      <c r="C6" s="2">
+        <v>-0.8891</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>Guanajuato, Mexico</t>
+        </is>
+      </c>
+      <c r="B7" s="2">
+        <v>21.019</v>
+      </c>
+      <c r="C7" s="2">
+        <v>-101.2574</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>Indiana, USA</t>
+        </is>
+      </c>
+      <c r="B8" s="2">
+        <v>40.4237</v>
+      </c>
+      <c r="C8" s="2">
+        <v>-86.9212</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>Columbia, USA</t>
+        </is>
+      </c>
+      <c r="B9" s="2">
+        <v>38.9517</v>
+      </c>
+      <c r="C9" s="2">
+        <v>-92.3341</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>Illinois, USA</t>
+        </is>
+      </c>
+      <c r="B10" s="2">
+        <v>41.8708</v>
+      </c>
+      <c r="C10" s="2">
+        <v>-87.6505</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>Michigan, USA</t>
+        </is>
+      </c>
+      <c r="B11" s="2">
+        <v>42.2808</v>
+      </c>
+      <c r="C11" s="2">
+        <v>-83.743</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>Milan, Italy</t>
+        </is>
+      </c>
+      <c r="B12" s="2">
+        <v>45.4642</v>
+      </c>
+      <c r="C12" s="2">
+        <v>9.19</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>Lausanne, Switzerland</t>
+        </is>
+      </c>
+      <c r="B13" s="2">
+        <v>46.5191</v>
+      </c>
+      <c r="C13" s="2">
+        <v>6.5668</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>Budapest, Hungary</t>
+        </is>
+      </c>
+      <c r="B14" s="2">
+        <v>47.4979</v>
+      </c>
+      <c r="C14" s="2">
+        <v>19.0402</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>How to use: one row per place, written exactly as in the place column of the other sheets. lat/lon are the coordinates of the pin on the homepage map (right-click a spot in Google Maps to copy them). A place with no row here is left off the map.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Short CV: one-page PDF with selected courses; button reads Short CV
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/cv/cv.xlsx
+++ b/cv/cv.xlsx
@@ -798,7 +798,7 @@
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>no</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
@@ -8531,7 +8531,11 @@
       </c>
       <c r="H3" s="2" t="inlineStr"/>
       <c r="I3" s="2" t="inlineStr"/>
-      <c r="J3" s="2" t="inlineStr"/>
+      <c r="J3" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
@@ -8563,7 +8567,11 @@
       <c r="G4" s="2" t="inlineStr"/>
       <c r="H4" s="2" t="inlineStr"/>
       <c r="I4" s="2" t="inlineStr"/>
-      <c r="J4" s="2" t="inlineStr"/>
+      <c r="J4" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
@@ -8635,7 +8643,11 @@
       <c r="G6" s="2" t="inlineStr"/>
       <c r="H6" s="2" t="inlineStr"/>
       <c r="I6" s="2" t="inlineStr"/>
-      <c r="J6" s="2" t="inlineStr"/>
+      <c r="J6" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="3" t="inlineStr">

</xml_diff>

<commit_message>
CV: pdf_title column; PDF calls the courses "A selection of other activities"
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/cv/cv.xlsx
+++ b/cv/cv.xlsx
@@ -436,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H12"/>
+  <dimension ref="A1:I12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -447,6 +447,7 @@
     <col width="14" customWidth="1" min="6" max="6"/>
     <col width="14" customWidth="1" min="7" max="7"/>
     <col width="15" customWidth="1" min="8" max="8"/>
+    <col width="32" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -490,6 +491,11 @@
           <t>web_collapsed</t>
         </is>
       </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>pdf_title</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -809,6 +815,11 @@
       <c r="H10" t="inlineStr">
         <is>
           <t>yes</t>
+        </is>
+      </c>
+      <c r="I10" s="2" t="inlineStr">
+        <is>
+          <t>A selection of other activities</t>
         </is>
       </c>
     </row>
@@ -823,7 +834,7 @@
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>How to use: sections appear in this order. type = list (rows from the sheet with the same name), text (the text column) or events (rows of the Events sheet with this contribution). web/pdf = yes/no. details_in_pdf = no hides the talk/poster title (or the details column) in the PDF. In the other sheets, put older entries first and add new ones at the bottom; the CV shows them newest first. web_collapsed = yes shows the section on the web page as a collapsible block, closed by default.</t>
+          <t>How to use: sections appear in this order. type = list (rows from the sheet with the same name), text (the text column) or events (rows of the Events sheet with this contribution). web/pdf = yes/no. details_in_pdf = no hides the talk/poster title (or the details column) in the PDF. In the other sheets, put older entries first and add new ones at the bottom; the CV shows them newest first. pdf_title = a different section title for the PDF (blank: the same as on the web). web_collapsed = yes shows the section on the web page as a collapsible block, closed by default.</t>
         </is>
       </c>
       <c r="B12" s="2" t="n"/>

</xml_diff>